<commit_message>
Activity Plan: per-class checkboxes — each row is one combined-session group
- Each Activity Plan row now defines one combination: Activity |
  Allowed Periods | tick the classes that attend together (Yes/blank in
  Excel, real checkboxes in the dashboard). Add rows for more groups;
  a class ticked in no row is unrestricted and not combined.
- Windows are per (activity, class) from the row the class is ticked in;
  legacy text labels (Primary/...) still parse as sub-groups.
- Workbooks rebuilt: 2 P.E.T rows (junior/senior ticks, periods 6,7)
  + open Karate row. Dashboard editor uses CheckboxColumn per class.
- Duplicate tick across rows -> warning, first row wins.
- NRCS regenerated: OPTIMAL, audit pass; Group 1 = 4 combined sessions
  (minimum), Group 2 = 1 shared session. Save->auto-commit verified
  end-to-end (commit 77bec7d came from the dashboard itself).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NRHS/Requirements/NRHS_Information.xlsx
+++ b/NRHS/Requirements/NRHS_Information.xlsx
@@ -3245,31 +3245,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="22" t="inlineStr">
         <is>
-          <t>Activity Plan</t>
+          <t>Activity Plan  (each row = one combined session group; tick the classes that attend together)</t>
         </is>
       </c>
     </row>
@@ -3368,82 +3368,66 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Primary</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Primary</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Primary</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Primary</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Primary</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Primary</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Primary</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Primary</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Primary</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Secondary</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Secondary</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Secondary</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>Secondary</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Secondary</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Karate</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
+          <t>P.E.T</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>6,7</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
@@ -3453,11 +3437,53 @@
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Karate</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
NRHS: dashboard edit of information workbook (23 Jul 2026 10:12)
</commit_message>
<xml_diff>
--- a/NRHS/Requirements/NRHS_Information.xlsx
+++ b/NRHS/Requirements/NRHS_Information.xlsx
@@ -2716,7 +2716,11 @@
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Leisure</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
           <t>Lunch Break</t>

</xml_diff>

<commit_message>
NRHS: dashboard edit of information workbook (23 Jul 2026 10:43)
</commit_message>
<xml_diff>
--- a/NRHS/Requirements/NRHS_Information.xlsx
+++ b/NRHS/Requirements/NRHS_Information.xlsx
@@ -939,10 +939,10 @@
         <v>4</v>
       </c>
       <c r="N11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
@@ -1086,10 +1086,10 @@
         <v>2</v>
       </c>
       <c r="N14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -1299,7 +1299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2036,6 +2036,83 @@
       </c>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>P.E.T</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>BHAVANI</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>BHAVANI</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>BHAVANI</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>BHAVANI</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>BHAVANI</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>BHAVANI</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>BHAVANI</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>BHAVANI</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>BHAVANI</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>BHAVANI</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>BHAVANI</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>BHAVANI</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>BHAVANI</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>BHAVANI</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
NRHS: dashboard edit of information workbook (23 Jul 2026 10:48)
</commit_message>
<xml_diff>
--- a/NRHS/Requirements/NRHS_Information.xlsx
+++ b/NRHS/Requirements/NRHS_Information.xlsx
@@ -2365,7 +2365,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3007,6 +3007,47 @@
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>JAYA LAKSHMI</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>MUST</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Lunch Break</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Leisure</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Leisure</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Leisure</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Leisure</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
NRHS: dashboard edit of information workbook (23 Jul 2026 10:49)
</commit_message>
<xml_diff>
--- a/NRHS/Requirements/NRHS_Information.xlsx
+++ b/NRHS/Requirements/NRHS_Information.xlsx
@@ -3408,16 +3408,8 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">

</xml_diff>

<commit_message>
NRHS: feasible workbook + generated timetable
- Fix JAYA LAKSHMI leisure typos (free P5/P6/P7 so she can teach UKG(B))
- P.E.T = 1 for Classes 3-8 (per request)
- Loosen P.E.T Activity-Plan period pins (keep days + Karate Thu P6): senior
  classes' afternoons are fully locked by Riya/Sunitha/Gowtham, so P.E.T can't
  stay afternoon-only and must use morning slots
- Regenerated NRHS_Timetable_Final.xlsx/.pdf; audit ALL PASS (597 slots)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NRHS/Requirements/NRHS_Information.xlsx
+++ b/NRHS/Requirements/NRHS_Information.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Weekly Period Plan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Teacher Allotment" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Period 1 teacher allotment" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Teacher Leisure Plan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Activity Plan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Period Plan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teacher Allotment" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Period 1 teacher allotment" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teacher Leisure Plan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Plan" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1068,22 +1068,22 @@
         <v>4</v>
       </c>
       <c r="H14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N14" t="n">
         <v>1</v>
@@ -1264,22 +1264,22 @@
         <v>42</v>
       </c>
       <c r="H18" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I18" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J18" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K18" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L18" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M18" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="N18" t="n">
         <v>47</v>
@@ -1469,7 +1469,6 @@
           <t>HINDI</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>BIJILI</t>
@@ -1741,11 +1740,6 @@
           <t>K.ESWAR</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1753,15 +1747,6 @@
           <t>PHYSICS</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>K.ESWAR</t>
@@ -1794,15 +1779,6 @@
           <t>CHEMISTRY</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>K.ESWAR</t>
@@ -1835,15 +1811,6 @@
           <t>BIOLOGY</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>S.GAYATHRI</t>
@@ -1876,12 +1843,6 @@
           <t>SOCIAL</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>R.KAMALA</t>
@@ -1929,9 +1890,6 @@
           <t>COMPUTER</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>VINAY</t>
@@ -1977,8 +1935,6 @@
           <t>VINAY</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1986,9 +1942,6 @@
           <t>G.K</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>CHANDRAKALA</t>
@@ -2034,8 +1987,6 @@
           <t>ESWAR</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2350,9 +2301,6 @@
           <t>Chandini</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2468,10 +2416,6 @@
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2509,10 +2453,6 @@
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2525,9 +2465,6 @@
           <t>MUST</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>Leisure</t>
@@ -2600,9 +2537,6 @@
           <t>Leisure</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2615,19 +2549,11 @@
           <t>BEST</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2640,19 +2566,11 @@
           <t>BEST</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2665,19 +2583,11 @@
           <t>BEST</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2690,19 +2600,11 @@
           <t>BEST</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2715,19 +2617,11 @@
           <t>BEST</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2740,19 +2634,11 @@
           <t>BEST</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2765,19 +2651,11 @@
           <t>BEST</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2790,9 +2668,6 @@
           <t>BEST</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>Leisure</t>
@@ -2803,10 +2678,6 @@
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2819,19 +2690,11 @@
           <t>BEST</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2844,19 +2707,11 @@
           <t>BEST</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2869,19 +2724,11 @@
           <t>BEST</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2894,19 +2741,11 @@
           <t>BEST</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2919,19 +2758,11 @@
           <t>BEST</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2944,19 +2775,11 @@
           <t>BEST</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2969,19 +2792,11 @@
           <t>BEST</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2994,19 +2809,11 @@
           <t>BEST</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3019,28 +2826,9 @@
           <t>MUST</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
           <t>Lunch Break</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Leisure</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>Leisure</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>Leisure</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -3168,11 +2956,6 @@
           <t>MON,WED,FRI</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3188,17 +2971,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3211,14 +2983,6 @@
           <t>MON,WED,FRI</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3234,14 +2998,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3254,17 +3010,6 @@
           <t>TUE</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3285,10 +3030,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3301,21 +3042,6 @@
           <t>TUE</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3348,25 +3074,6 @@
           <t>TUE</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3379,20 +3086,6 @@
           <t>SAT</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3408,8 +3101,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3427,9 +3118,6 @@
           <t>6</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3475,8 +3163,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3489,16 +3175,6 @@
           <t>SAT</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3519,11 +3195,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>